<commit_message>
criada fora da main uma função que salva os dados em excel e ajusta lagura
</commit_message>
<xml_diff>
--- a/xlsx_tratado/dados_jogo.xlsx
+++ b/xlsx_tratado/dados_jogo.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="jogo ID3240220" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="jogo ID1145350" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -416,9 +416,9 @@
   <dimension ref="A1:AR2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
@@ -430,25 +430,25 @@
     <col width="17" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
-    <col width="34" customWidth="1" min="15" max="15"/>
-    <col width="37" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
     <col width="15" customWidth="1" min="17" max="17"/>
-    <col width="70" customWidth="1" min="18" max="18"/>
+    <col width="58" customWidth="1" min="18" max="18"/>
     <col width="17" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="43" customWidth="1" min="21" max="21"/>
+    <col width="19" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
     <col width="15" customWidth="1" min="22" max="22"/>
-    <col width="72" customWidth="1" min="23" max="23"/>
+    <col width="56" customWidth="1" min="23" max="23"/>
     <col width="17" customWidth="1" min="24" max="24"/>
-    <col width="15" customWidth="1" min="25" max="25"/>
-    <col width="15" customWidth="1" min="26" max="26"/>
+    <col width="19" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
     <col width="16" customWidth="1" min="27" max="27"/>
-    <col width="15" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
     <col width="18" customWidth="1" min="29" max="29"/>
-    <col width="15" customWidth="1" min="30" max="30"/>
-    <col width="15" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="14" customWidth="1" min="31" max="31"/>
     <col width="16" customWidth="1" min="32" max="32"/>
-    <col width="15" customWidth="1" min="33" max="33"/>
+    <col width="14" customWidth="1" min="33" max="33"/>
     <col width="18" customWidth="1" min="34" max="34"/>
     <col width="15" customWidth="1" min="35" max="35"/>
     <col width="15" customWidth="1" min="36" max="36"/>
@@ -687,15 +687,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Grand Theft Auto V Enhanced</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
+          <t>Hades II</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ação, Aventura, Corridas</t>
+          <t>Ação, Indie, RPG</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -704,41 +706,44 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>14990</v>
+        <v>8899</v>
       </c>
       <c r="F2" t="n">
-        <v>14990</v>
+        <v>8899</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>R$ 149,90</t>
+          <t>R$ 88,99</t>
         </is>
       </c>
       <c r="J2" t="n">
         <v>1</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
       </c>
+      <c r="M2" t="n">
+        <v>94</v>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>4 mar. 2025</t>
+          <t>25 set. 2025</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Windows 10 (latest service pack)</t>
+          <t>Windows 10 64-bit</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Intel® Core™ i7-4770 | AMD FX™-9590</t>
+          <t>Dual Core 2.4 GHz</t>
         </is>
       </c>
       <c r="Q2" t="n">
@@ -746,20 +751,20 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>NVIDIA GeForce® GTX 1630 (4GB VRAM) | AMD Radeon™ RX 6400 (4GB VRAM)</t>
+          <t>GeForce GTX 950, Radeon R7 360, or Intel HD Graphics 630</t>
         </is>
       </c>
       <c r="S2" t="n">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>Windows 11</t>
+          <t>Windows 10 64-bit</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Intel® Core™ i5-9600K | AMD Ryzen™ 5 3600</t>
+          <t>Quad Core 2.4ghz</t>
         </is>
       </c>
       <c r="V2" t="n">
@@ -767,61 +772,53 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>NVIDIA GeForce® RTX 3060 (8GB VRAM) | AMD Radeon™ RX 6600XT (8GB VRAM)</t>
+          <t>GeForce RTX 2060, Radeon RX 5600 XT, or Intel Arc A580</t>
         </is>
       </c>
       <c r="X2" t="n">
-        <v>105</v>
+        <v>11</v>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Não suportado</t>
+          <t>macOS 12 or newer</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Não suportado</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>Não suportado</t>
-        </is>
+          <t>Apple M1</t>
+        </is>
+      </c>
+      <c r="AA2" t="n">
+        <v>8</v>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Não suportado</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>Não suportado</t>
-        </is>
+          <t>Apple M1</t>
+        </is>
+      </c>
+      <c r="AC2" t="n">
+        <v>11</v>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>Não suportado</t>
+          <t>macOS 15</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>Não suportado</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>Não suportado</t>
-        </is>
+          <t>Apple M1 Pro</t>
+        </is>
+      </c>
+      <c r="AF2" t="n">
+        <v>16</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>Não suportado</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>Não suportado</t>
-        </is>
+          <t>Apple M1 Pro</t>
+        </is>
+      </c>
+      <c r="AH2" t="n">
+        <v>11</v>
       </c>
       <c r="AI2" t="inlineStr">
         <is>

</xml_diff>